<commit_message>
classification of climate relevant businesses, test BERTopic
</commit_message>
<xml_diff>
--- a/french_dictionary_curated.xlsx
+++ b/french_dictionary_curated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sile9\Documents\projects\parldebates_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C968BD2-4CD1-43CC-A26A-E69B3A0C62B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74475831-6296-44F0-BCC2-DF64CC3F8364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="61">
   <si>
     <t>keyword_french</t>
   </si>
@@ -130,33 +130,12 @@
     <t>deforestation</t>
   </si>
   <si>
-    <t>écologiques</t>
-  </si>
-  <si>
-    <t>environmentally friendly</t>
-  </si>
-  <si>
     <t>électricité</t>
   </si>
   <si>
     <t>electricity</t>
   </si>
   <si>
-    <t>émission</t>
-  </si>
-  <si>
-    <t>broadcast</t>
-  </si>
-  <si>
-    <t>émissions</t>
-  </si>
-  <si>
-    <t>emissions</t>
-  </si>
-  <si>
-    <t>énergétique</t>
-  </si>
-  <si>
     <t>energy</t>
   </si>
   <si>
@@ -217,13 +196,13 @@
     <t>réchauffement</t>
   </si>
   <si>
-    <t>warming</t>
-  </si>
-  <si>
     <t>renouvelables</t>
   </si>
   <si>
     <t>renewables</t>
+  </si>
+  <si>
+    <t>heating</t>
   </si>
 </sst>
 </file>
@@ -557,13 +536,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.21875" customWidth="1"/>
+    <col min="1" max="1" width="30.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -571,7 +550,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -579,7 +558,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -587,7 +566,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -595,7 +574,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -603,7 +582,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -611,7 +590,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -619,7 +598,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -627,7 +606,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -635,7 +614,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -643,7 +622,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -651,7 +630,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -659,7 +638,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -667,7 +646,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -675,7 +654,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -683,7 +662,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -691,7 +670,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -699,7 +678,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -707,7 +686,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -715,7 +694,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -723,7 +702,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -731,23 +710,23 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" t="s">
         <v>38</v>
       </c>
-      <c r="B22" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" t="s">
         <v>40</v>
       </c>
-      <c r="B23" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -755,7 +734,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>44</v>
       </c>
@@ -763,47 +742,47 @@
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>46</v>
       </c>
       <c r="B26" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>48</v>
       </c>
       <c r="B27" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B28" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B29" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" t="s">
         <v>53</v>
       </c>
-      <c r="B30" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>55</v>
       </c>
@@ -811,52 +790,20 @@
         <v>56</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>57</v>
       </c>
       <c r="B32" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
         <v>59</v>
-      </c>
-      <c r="B33" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>61</v>
-      </c>
-      <c r="B34" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>62</v>
-      </c>
-      <c r="B35" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>64</v>
-      </c>
-      <c r="B36" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>66</v>
-      </c>
-      <c r="B37" t="s">
-        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>